<commit_message>
docs: PERT calculation added
</commit_message>
<xml_diff>
--- a/сводная таблица оценок и PERT.xlsx
+++ b/сводная таблица оценок и PERT.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/1f1cfff57e867f98/ВГУ/4 курс - 7 семестр/Управление проектами/photo-studio/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="116" documentId="11_AD4DF75460589B3ACB72848187DB6FA05ADEDD8E" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{A7D7BFA6-7C56-46B1-9D92-9B5B73F7A0A9}"/>
+  <xr:revisionPtr revIDLastSave="353" documentId="11_AD4DF75460589B3ACB72848187DB6FA05ADEDD8E" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{59DEC8DC-2621-486D-A258-F8DC841BE7D4}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Оценки пакетов ИСР" sheetId="1" r:id="rId1"/>
@@ -37,7 +37,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="114" uniqueCount="82">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="200" uniqueCount="143">
   <si>
     <t>Код ИСР</t>
   </si>
@@ -210,6 +210,9 @@
     <t xml:space="preserve">	1.2.1</t>
   </si>
   <si>
+    <t>1.2.1</t>
+  </si>
+  <si>
     <t>1.2.2</t>
   </si>
   <si>
@@ -283,6 +286,186 @@
   </si>
   <si>
     <t xml:space="preserve">	1.1.1</t>
+  </si>
+  <si>
+    <t>АНАЛИЗ СЕТЕВОГО ГРАФИКА И РАСЧЁТ МЕТОДОМ PERT</t>
+  </si>
+  <si>
+    <t>1. Параметры критического пути</t>
+  </si>
+  <si>
+    <t>Критическая цепочка пакетов ИСР:</t>
+  </si>
+  <si>
+    <t>1.1.1 → 2.1.2 → 2.2.2 → 3.1.1 → 3.1.2 → 3.2.1 → 3.2.2 → 3.3.1 → 3.3.2 → 4.1.1 → 4.1.2 → 4.2.2</t>
+  </si>
+  <si>
+    <t>Непрерывная цепочка самых длительных работ</t>
+  </si>
+  <si>
+    <t>Длительность критического пути (T_cp), ч:</t>
+  </si>
+  <si>
+    <t>Дисперсия критического пути (σ^2_cp):</t>
+  </si>
+  <si>
+    <t>Стандартное отклонение (σ_cp), ч:</t>
+  </si>
+  <si>
+    <t>Параметр</t>
+  </si>
+  <si>
+    <t>Формула / Значение в Excel</t>
+  </si>
+  <si>
+    <t>Пояснение</t>
+  </si>
+  <si>
+    <t>Сумма t_e критических работ</t>
+  </si>
+  <si>
+    <t>Сумма дисперсий</t>
+  </si>
+  <si>
+    <t>2. Оценка вероятности сдачи до конца семестра</t>
+  </si>
+  <si>
+    <t>Лимит времени критической цепочки на семестр</t>
+  </si>
+  <si>
+    <t>Вывод по срокам:</t>
+  </si>
+  <si>
+    <t>Проект реализуем в срок с вероятностью 98%. Урезание скоупа не требуется.</t>
+  </si>
+  <si>
+    <t>Директивный срок команды (T_dir), ч:</t>
+  </si>
+  <si>
+    <t>Ожидаемая длительность критического пути (T_cp), ч:</t>
+  </si>
+  <si>
+    <t>Z -показатель (нормированное отклонение):</t>
+  </si>
+  <si>
+    <t>Вероятность уложиться в срок (P):</t>
+  </si>
+  <si>
+    <t>Формула (T_dir−T_cp)/σ_cp</t>
+  </si>
+  <si>
+    <t>3. Сверка с ограничениями Устава</t>
+  </si>
+  <si>
+    <t>Общий фонд времени команды по Уставу, ч:</t>
+  </si>
+  <si>
+    <t>Суммарная плановая трудоёмкость 25 пакетов, ч:</t>
+  </si>
+  <si>
+    <t>Буфер рабочего времени команды, ч:</t>
+  </si>
+  <si>
+    <t>Утвержденный фонд оплаты труда по Уставу, ₽:</t>
+  </si>
+  <si>
+    <t>Плановая стоимость работ базового плана, ₽:</t>
+  </si>
+  <si>
+    <t>Экономия / Резерв по бюджету, ₽:</t>
+  </si>
+  <si>
+    <t xml:space="preserve">	5 человек × 6 ч/нед × 14 недель</t>
+  </si>
+  <si>
+    <t>Ссылка на ИТОГО Листа 1</t>
+  </si>
+  <si>
+    <t>Запас времени команды: 33 ч (8,5%)</t>
+  </si>
+  <si>
+    <t>Лимит ФОТ из Устава (п. 5.4)</t>
+  </si>
+  <si>
+    <t>Ссылка на ИТОГО Листа 1 (209 850 ₽)</t>
+  </si>
+  <si>
+    <t>Экономия фонда: 12 750 ₽</t>
+  </si>
+  <si>
+    <t>4. Резервы времени некритических пакетов работ</t>
+  </si>
+  <si>
+    <t>A (Пакет ИСР)</t>
+  </si>
+  <si>
+    <t>B (Название пакета)</t>
+  </si>
+  <si>
+    <t>Код</t>
+  </si>
+  <si>
+    <t>ES</t>
+  </si>
+  <si>
+    <t>LS</t>
+  </si>
+  <si>
+    <t>TF</t>
+  </si>
+  <si>
+    <t>FF</t>
+  </si>
+  <si>
+    <t>4 ч</t>
+  </si>
+  <si>
+    <t>5 ч</t>
+  </si>
+  <si>
+    <t>11 ч</t>
+  </si>
+  <si>
+    <t>7 ч</t>
+  </si>
+  <si>
+    <t>Макеты интерфейса (дизайн)</t>
+  </si>
+  <si>
+    <t>13 ч</t>
+  </si>
+  <si>
+    <t>Раздел «Мои брони»</t>
+  </si>
+  <si>
+    <t>17 ч</t>
+  </si>
+  <si>
+    <t>22 ч</t>
+  </si>
+  <si>
+    <t>19 ч</t>
+  </si>
+  <si>
+    <t>C (t_e, ч)</t>
+  </si>
+  <si>
+    <t>D (Ранний старт ES)</t>
+  </si>
+  <si>
+    <t>E (Поздний старт LS)</t>
+  </si>
+  <si>
+    <t>F (Полный резерв TF)</t>
+  </si>
+  <si>
+    <t>G (Свободный резерв FF)</t>
+  </si>
+  <si>
+    <t>2.2.1</t>
+  </si>
+  <si>
+    <t>t_e</t>
   </si>
 </sst>
 </file>
@@ -292,7 +475,14 @@
   <numFmts count="1">
     <numFmt numFmtId="6" formatCode="#,##0\ &quot;₽&quot;;[Red]\-#,##0\ &quot;₽&quot;"/>
   </numFmts>
-  <fonts count="2" x14ac:knownFonts="1">
+  <fonts count="5" x14ac:knownFonts="1">
+    <font>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -307,8 +497,22 @@
       <family val="2"/>
       <scheme val="minor"/>
     </font>
+    <font>
+      <sz val="8"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="14"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
   </fonts>
-  <fills count="3">
+  <fills count="5">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -321,8 +525,20 @@
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="4" tint="0.39997558519241921"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="9" tint="0.59999389629810485"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
   </fills>
-  <borders count="2">
+  <borders count="5">
     <border>
       <left/>
       <right/>
@@ -345,42 +561,135 @@
       </bottom>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin">
+        <color indexed="64"/>
+      </left>
+      <right/>
+      <top style="thin">
+        <color indexed="64"/>
+      </top>
+      <bottom style="thin">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right/>
+      <top style="thin">
+        <color indexed="64"/>
+      </top>
+      <bottom style="thin">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="thin">
+        <color indexed="64"/>
+      </right>
+      <top style="thin">
+        <color indexed="64"/>
+      </top>
+      <bottom style="thin">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
-  <cellStyleXfs count="1">
+  <cellStyleXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
+    <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="10">
+  <cellXfs count="28">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="3" fontId="1" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="3" fontId="2" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="6" fontId="1" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="6" fontId="2" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+    <xf numFmtId="49" fontId="2" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="49" fontId="1" fillId="2" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="49" fontId="2" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="49" fontId="1" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="2" fontId="2" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="49" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+    <xf numFmtId="49" fontId="2" fillId="2" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="3" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="3" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="3" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="9" fontId="2" fillId="0" borderId="1" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="3" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="3" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="3" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="49" fontId="2" fillId="4" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="49" fontId="2" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
   </cellXfs>
-  <cellStyles count="1">
+  <cellStyles count="2">
     <cellStyle name="Обычный" xfId="0" builtinId="0"/>
+    <cellStyle name="Процентный" xfId="1" builtinId="5"/>
   </cellStyles>
   <dxfs count="0"/>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
@@ -661,57 +970,57 @@
   <dimension ref="A1:K27"/>
   <sheetFormatPr defaultRowHeight="18.75" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="10.85546875" style="8" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="46" style="5" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="18.85546875" style="5" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="23.28515625" style="8" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="8.42578125" style="5" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="8.5703125" style="5" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="8.42578125" style="5" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="8.28515625" style="5" bestFit="1" customWidth="1"/>
-    <col min="9" max="9" width="20.140625" style="8" bestFit="1" customWidth="1"/>
-    <col min="10" max="10" width="15" style="5" bestFit="1" customWidth="1"/>
-    <col min="11" max="11" width="17.140625" style="5" bestFit="1" customWidth="1"/>
-    <col min="12" max="16384" width="9.140625" style="5"/>
+    <col min="1" max="1" width="10.85546875" style="6" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="46" style="4" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="18.85546875" style="4" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="23.28515625" style="6" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="8.42578125" style="4" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="8.5703125" style="4" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="8.42578125" style="4" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="8.28515625" style="4" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="20.140625" style="6" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="15" style="4" bestFit="1" customWidth="1"/>
+    <col min="11" max="11" width="17.140625" style="4" bestFit="1" customWidth="1"/>
+    <col min="12" max="16384" width="9.140625" style="4"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A1" s="6" t="s">
+    <row r="1" spans="1:11" s="10" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A1" s="8" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="4" t="s">
+      <c r="B1" s="9" t="s">
         <v>1</v>
       </c>
-      <c r="C1" s="4" t="s">
+      <c r="C1" s="9" t="s">
         <v>2</v>
       </c>
-      <c r="D1" s="6" t="s">
+      <c r="D1" s="8" t="s">
         <v>3</v>
       </c>
-      <c r="E1" s="4" t="s">
+      <c r="E1" s="9" t="s">
         <v>45</v>
       </c>
-      <c r="F1" s="4" t="s">
+      <c r="F1" s="9" t="s">
         <v>49</v>
       </c>
-      <c r="G1" s="4" t="s">
+      <c r="G1" s="9" t="s">
         <v>46</v>
       </c>
-      <c r="H1" s="4" t="s">
+      <c r="H1" s="9" t="s">
         <v>48</v>
       </c>
-      <c r="I1" s="6" t="s">
+      <c r="I1" s="8" t="s">
         <v>47</v>
       </c>
-      <c r="J1" s="4" t="s">
+      <c r="J1" s="9" t="s">
         <v>4</v>
       </c>
-      <c r="K1" s="4" t="s">
+      <c r="K1" s="9" t="s">
         <v>5</v>
       </c>
     </row>
     <row r="2" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A2" s="7" t="s">
+      <c r="A2" s="5" t="s">
         <v>50</v>
       </c>
       <c r="B2" s="1" t="s">
@@ -720,7 +1029,7 @@
       <c r="C2" s="1" t="s">
         <v>7</v>
       </c>
-      <c r="D2" s="7" t="s">
+      <c r="D2" s="5" t="s">
         <v>8</v>
       </c>
       <c r="E2" s="1">
@@ -736,7 +1045,7 @@
         <f>(E2 + 4*F2 + G2) / 6</f>
         <v>19</v>
       </c>
-      <c r="I2" s="9">
+      <c r="I2" s="7">
         <f>((G2 - E2) / 6)^2</f>
         <v>5.4444444444444455</v>
       </c>
@@ -749,7 +1058,7 @@
       </c>
     </row>
     <row r="3" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A3" s="7" t="s">
+      <c r="A3" s="5" t="s">
         <v>52</v>
       </c>
       <c r="B3" s="1" t="s">
@@ -758,7 +1067,7 @@
       <c r="C3" s="1" t="s">
         <v>7</v>
       </c>
-      <c r="D3" s="7" t="s">
+      <c r="D3" s="5" t="s">
         <v>10</v>
       </c>
       <c r="E3" s="1">
@@ -774,7 +1083,7 @@
         <f t="shared" ref="H3:H27" si="0">(E3 + 4*F3 + G3) / 6</f>
         <v>17</v>
       </c>
-      <c r="I3" s="9">
+      <c r="I3" s="7">
         <f t="shared" ref="I3:I26" si="1">((G3 - E3) / 6)^2</f>
         <v>5.4444444444444455</v>
       </c>
@@ -787,7 +1096,7 @@
       </c>
     </row>
     <row r="4" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A4" s="7" t="s">
+      <c r="A4" s="5" t="s">
         <v>55</v>
       </c>
       <c r="B4" s="1" t="s">
@@ -796,8 +1105,8 @@
       <c r="C4" s="1" t="s">
         <v>7</v>
       </c>
-      <c r="D4" s="7" t="s">
-        <v>81</v>
+      <c r="D4" s="5" t="s">
+        <v>82</v>
       </c>
       <c r="E4" s="1">
         <v>8</v>
@@ -812,7 +1121,7 @@
         <f t="shared" si="0"/>
         <v>11</v>
       </c>
-      <c r="I4" s="9">
+      <c r="I4" s="7">
         <f t="shared" si="1"/>
         <v>2.7777777777777781</v>
       </c>
@@ -825,7 +1134,7 @@
       </c>
     </row>
     <row r="5" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A5" s="7" t="s">
+      <c r="A5" s="5" t="s">
         <v>56</v>
       </c>
       <c r="B5" s="1" t="s">
@@ -834,8 +1143,8 @@
       <c r="C5" s="1" t="s">
         <v>13</v>
       </c>
-      <c r="D5" s="7" t="s">
-        <v>81</v>
+      <c r="D5" s="5" t="s">
+        <v>82</v>
       </c>
       <c r="E5" s="1">
         <v>10</v>
@@ -850,7 +1159,7 @@
         <f t="shared" si="0"/>
         <v>15</v>
       </c>
-      <c r="I5" s="9">
+      <c r="I5" s="7">
         <f t="shared" si="1"/>
         <v>5.4444444444444455</v>
       </c>
@@ -863,8 +1172,8 @@
       </c>
     </row>
     <row r="6" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A6" s="7" t="s">
-        <v>57</v>
+      <c r="A6" s="5" t="s">
+        <v>58</v>
       </c>
       <c r="B6" s="1" t="s">
         <v>14</v>
@@ -872,7 +1181,7 @@
       <c r="C6" s="1" t="s">
         <v>13</v>
       </c>
-      <c r="D6" s="7" t="s">
+      <c r="D6" s="5" t="s">
         <v>15</v>
       </c>
       <c r="E6" s="1">
@@ -888,7 +1197,7 @@
         <f t="shared" si="0"/>
         <v>15</v>
       </c>
-      <c r="I6" s="9">
+      <c r="I6" s="7">
         <f t="shared" si="1"/>
         <v>5.4444444444444455</v>
       </c>
@@ -901,8 +1210,8 @@
       </c>
     </row>
     <row r="7" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A7" s="7" t="s">
-        <v>60</v>
+      <c r="A7" s="5" t="s">
+        <v>61</v>
       </c>
       <c r="B7" s="1" t="s">
         <v>16</v>
@@ -910,8 +1219,8 @@
       <c r="C7" s="1" t="s">
         <v>7</v>
       </c>
-      <c r="D7" s="7" t="s">
-        <v>80</v>
+      <c r="D7" s="5" t="s">
+        <v>81</v>
       </c>
       <c r="E7" s="1">
         <v>12</v>
@@ -926,7 +1235,7 @@
         <f t="shared" si="0"/>
         <v>17</v>
       </c>
-      <c r="I7" s="9">
+      <c r="I7" s="7">
         <f t="shared" si="1"/>
         <v>5.4444444444444455</v>
       </c>
@@ -939,7 +1248,7 @@
       </c>
     </row>
     <row r="8" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A8" s="7" t="s">
+      <c r="A8" s="5" t="s">
         <v>53</v>
       </c>
       <c r="B8" s="1" t="s">
@@ -948,7 +1257,7 @@
       <c r="C8" s="1" t="s">
         <v>18</v>
       </c>
-      <c r="D8" s="7" t="s">
+      <c r="D8" s="5" t="s">
         <v>8</v>
       </c>
       <c r="E8" s="1">
@@ -964,7 +1273,7 @@
         <f t="shared" si="0"/>
         <v>15</v>
       </c>
-      <c r="I8" s="9">
+      <c r="I8" s="7">
         <f t="shared" si="1"/>
         <v>5.4444444444444455</v>
       </c>
@@ -977,8 +1286,8 @@
       </c>
     </row>
     <row r="9" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A9" s="7" t="s">
-        <v>58</v>
+      <c r="A9" s="5" t="s">
+        <v>59</v>
       </c>
       <c r="B9" s="1" t="s">
         <v>19</v>
@@ -986,7 +1295,7 @@
       <c r="C9" s="1" t="s">
         <v>18</v>
       </c>
-      <c r="D9" s="7" t="s">
+      <c r="D9" s="5" t="s">
         <v>20</v>
       </c>
       <c r="E9" s="1">
@@ -1002,7 +1311,7 @@
         <f t="shared" si="0"/>
         <v>19</v>
       </c>
-      <c r="I9" s="9">
+      <c r="I9" s="7">
         <f t="shared" si="1"/>
         <v>5.4444444444444455</v>
       </c>
@@ -1015,8 +1324,8 @@
       </c>
     </row>
     <row r="10" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A10" s="7" t="s">
-        <v>62</v>
+      <c r="A10" s="5" t="s">
+        <v>63</v>
       </c>
       <c r="B10" s="1" t="s">
         <v>21</v>
@@ -1024,8 +1333,8 @@
       <c r="C10" s="1" t="s">
         <v>22</v>
       </c>
-      <c r="D10" s="7" t="s">
-        <v>79</v>
+      <c r="D10" s="5" t="s">
+        <v>80</v>
       </c>
       <c r="E10" s="1">
         <v>22</v>
@@ -1040,7 +1349,7 @@
         <f t="shared" si="0"/>
         <v>30</v>
       </c>
-      <c r="I10" s="9">
+      <c r="I10" s="7">
         <f t="shared" si="1"/>
         <v>16</v>
       </c>
@@ -1053,7 +1362,7 @@
       </c>
     </row>
     <row r="11" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A11" s="7" t="s">
+      <c r="A11" s="5" t="s">
         <v>51</v>
       </c>
       <c r="B11" s="1" t="s">
@@ -1062,8 +1371,8 @@
       <c r="C11" s="1" t="s">
         <v>24</v>
       </c>
-      <c r="D11" s="7" t="s">
-        <v>58</v>
+      <c r="D11" s="5" t="s">
+        <v>59</v>
       </c>
       <c r="E11" s="1">
         <v>10</v>
@@ -1078,7 +1387,7 @@
         <f t="shared" si="0"/>
         <v>15</v>
       </c>
-      <c r="I11" s="9">
+      <c r="I11" s="7">
         <f t="shared" si="1"/>
         <v>5.4444444444444455</v>
       </c>
@@ -1091,8 +1400,8 @@
       </c>
     </row>
     <row r="12" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A12" s="7" t="s">
-        <v>61</v>
+      <c r="A12" s="5" t="s">
+        <v>62</v>
       </c>
       <c r="B12" s="1" t="s">
         <v>25</v>
@@ -1100,8 +1409,8 @@
       <c r="C12" s="1" t="s">
         <v>24</v>
       </c>
-      <c r="D12" s="7" t="s">
-        <v>78</v>
+      <c r="D12" s="5" t="s">
+        <v>79</v>
       </c>
       <c r="E12" s="1">
         <v>8</v>
@@ -1116,7 +1425,7 @@
         <f t="shared" si="0"/>
         <v>13</v>
       </c>
-      <c r="I12" s="9">
+      <c r="I12" s="7">
         <f t="shared" si="1"/>
         <v>5.4444444444444455</v>
       </c>
@@ -1129,8 +1438,8 @@
       </c>
     </row>
     <row r="13" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A13" s="7" t="s">
-        <v>63</v>
+      <c r="A13" s="5" t="s">
+        <v>64</v>
       </c>
       <c r="B13" s="1" t="s">
         <v>26</v>
@@ -1138,8 +1447,8 @@
       <c r="C13" s="1" t="s">
         <v>24</v>
       </c>
-      <c r="D13" s="7" t="s">
-        <v>77</v>
+      <c r="D13" s="5" t="s">
+        <v>78</v>
       </c>
       <c r="E13" s="1">
         <v>10</v>
@@ -1154,7 +1463,7 @@
         <f t="shared" si="0"/>
         <v>15</v>
       </c>
-      <c r="I13" s="9">
+      <c r="I13" s="7">
         <f t="shared" si="1"/>
         <v>5.4444444444444455</v>
       </c>
@@ -1167,8 +1476,8 @@
       </c>
     </row>
     <row r="14" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A14" s="7" t="s">
-        <v>64</v>
+      <c r="A14" s="5" t="s">
+        <v>65</v>
       </c>
       <c r="B14" s="1" t="s">
         <v>27</v>
@@ -1176,7 +1485,7 @@
       <c r="C14" s="1" t="s">
         <v>24</v>
       </c>
-      <c r="D14" s="7" t="s">
+      <c r="D14" s="5" t="s">
         <v>28</v>
       </c>
       <c r="E14" s="1">
@@ -1192,7 +1501,7 @@
         <f t="shared" si="0"/>
         <v>17</v>
       </c>
-      <c r="I14" s="9">
+      <c r="I14" s="7">
         <f t="shared" si="1"/>
         <v>5.4444444444444455</v>
       </c>
@@ -1205,8 +1514,8 @@
       </c>
     </row>
     <row r="15" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A15" s="7" t="s">
-        <v>65</v>
+      <c r="A15" s="5" t="s">
+        <v>66</v>
       </c>
       <c r="B15" s="1" t="s">
         <v>29</v>
@@ -1214,8 +1523,8 @@
       <c r="C15" s="1" t="s">
         <v>24</v>
       </c>
-      <c r="D15" s="7" t="s">
-        <v>76</v>
+      <c r="D15" s="5" t="s">
+        <v>77</v>
       </c>
       <c r="E15" s="1">
         <v>16</v>
@@ -1230,7 +1539,7 @@
         <f t="shared" si="0"/>
         <v>23</v>
       </c>
-      <c r="I15" s="9">
+      <c r="I15" s="7">
         <f t="shared" si="1"/>
         <v>9</v>
       </c>
@@ -1243,8 +1552,8 @@
       </c>
     </row>
     <row r="16" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A16" s="7" t="s">
-        <v>66</v>
+      <c r="A16" s="5" t="s">
+        <v>67</v>
       </c>
       <c r="B16" s="1" t="s">
         <v>30</v>
@@ -1252,8 +1561,8 @@
       <c r="C16" s="1" t="s">
         <v>24</v>
       </c>
-      <c r="D16" s="7" t="s">
-        <v>65</v>
+      <c r="D16" s="5" t="s">
+        <v>66</v>
       </c>
       <c r="E16" s="1">
         <v>10</v>
@@ -1268,7 +1577,7 @@
         <f t="shared" si="0"/>
         <v>15</v>
       </c>
-      <c r="I16" s="9">
+      <c r="I16" s="7">
         <f t="shared" si="1"/>
         <v>5.4444444444444455</v>
       </c>
@@ -1281,8 +1590,8 @@
       </c>
     </row>
     <row r="17" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A17" s="7" t="s">
-        <v>67</v>
+      <c r="A17" s="5" t="s">
+        <v>68</v>
       </c>
       <c r="B17" s="1" t="s">
         <v>31</v>
@@ -1290,8 +1599,8 @@
       <c r="C17" s="1" t="s">
         <v>24</v>
       </c>
-      <c r="D17" s="7" t="s">
-        <v>65</v>
+      <c r="D17" s="5" t="s">
+        <v>66</v>
       </c>
       <c r="E17" s="1">
         <v>14</v>
@@ -1306,7 +1615,7 @@
         <f t="shared" si="0"/>
         <v>20</v>
       </c>
-      <c r="I17" s="9">
+      <c r="I17" s="7">
         <f t="shared" si="1"/>
         <v>11.111111111111112</v>
       </c>
@@ -1319,8 +1628,8 @@
       </c>
     </row>
     <row r="18" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A18" s="7" t="s">
-        <v>68</v>
+      <c r="A18" s="5" t="s">
+        <v>69</v>
       </c>
       <c r="B18" s="1" t="s">
         <v>32</v>
@@ -1328,8 +1637,8 @@
       <c r="C18" s="1" t="s">
         <v>24</v>
       </c>
-      <c r="D18" s="7" t="s">
-        <v>67</v>
+      <c r="D18" s="5" t="s">
+        <v>68</v>
       </c>
       <c r="E18" s="1">
         <v>12</v>
@@ -1344,7 +1653,7 @@
         <f t="shared" si="0"/>
         <v>17</v>
       </c>
-      <c r="I18" s="9">
+      <c r="I18" s="7">
         <f t="shared" si="1"/>
         <v>5.4444444444444455</v>
       </c>
@@ -1357,7 +1666,7 @@
       </c>
     </row>
     <row r="19" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A19" s="7" t="s">
+      <c r="A19" s="5" t="s">
         <v>54</v>
       </c>
       <c r="B19" s="1" t="s">
@@ -1366,8 +1675,8 @@
       <c r="C19" s="1" t="s">
         <v>24</v>
       </c>
-      <c r="D19" s="7" t="s">
-        <v>67</v>
+      <c r="D19" s="5" t="s">
+        <v>68</v>
       </c>
       <c r="E19" s="1">
         <v>8</v>
@@ -1382,7 +1691,7 @@
         <f t="shared" si="0"/>
         <v>13</v>
       </c>
-      <c r="I19" s="9">
+      <c r="I19" s="7">
         <f t="shared" si="1"/>
         <v>5.4444444444444455</v>
       </c>
@@ -1395,8 +1704,8 @@
       </c>
     </row>
     <row r="20" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A20" s="7" t="s">
-        <v>69</v>
+      <c r="A20" s="5" t="s">
+        <v>70</v>
       </c>
       <c r="B20" s="1" t="s">
         <v>34</v>
@@ -1404,8 +1713,8 @@
       <c r="C20" s="1" t="s">
         <v>24</v>
       </c>
-      <c r="D20" s="7" t="s">
-        <v>75</v>
+      <c r="D20" s="5" t="s">
+        <v>76</v>
       </c>
       <c r="E20" s="1">
         <v>10</v>
@@ -1420,7 +1729,7 @@
         <f t="shared" si="0"/>
         <v>15</v>
       </c>
-      <c r="I20" s="9">
+      <c r="I20" s="7">
         <f t="shared" si="1"/>
         <v>5.4444444444444455</v>
       </c>
@@ -1433,8 +1742,8 @@
       </c>
     </row>
     <row r="21" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A21" s="7" t="s">
-        <v>70</v>
+      <c r="A21" s="5" t="s">
+        <v>71</v>
       </c>
       <c r="B21" s="1" t="s">
         <v>35</v>
@@ -1442,8 +1751,8 @@
       <c r="C21" s="1" t="s">
         <v>24</v>
       </c>
-      <c r="D21" s="7" t="s">
-        <v>75</v>
+      <c r="D21" s="5" t="s">
+        <v>76</v>
       </c>
       <c r="E21" s="1">
         <v>6</v>
@@ -1458,7 +1767,7 @@
         <f t="shared" si="0"/>
         <v>9</v>
       </c>
-      <c r="I21" s="9">
+      <c r="I21" s="7">
         <f t="shared" si="1"/>
         <v>2.7777777777777781</v>
       </c>
@@ -1471,8 +1780,8 @@
       </c>
     </row>
     <row r="22" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A22" s="7" t="s">
-        <v>71</v>
+      <c r="A22" s="5" t="s">
+        <v>72</v>
       </c>
       <c r="B22" s="1" t="s">
         <v>36</v>
@@ -1480,8 +1789,8 @@
       <c r="C22" s="1" t="s">
         <v>24</v>
       </c>
-      <c r="D22" s="7" t="s">
-        <v>75</v>
+      <c r="D22" s="5" t="s">
+        <v>76</v>
       </c>
       <c r="E22" s="1">
         <v>6</v>
@@ -1496,7 +1805,7 @@
         <f t="shared" si="0"/>
         <v>9</v>
       </c>
-      <c r="I22" s="9">
+      <c r="I22" s="7">
         <f t="shared" si="1"/>
         <v>2.7777777777777781</v>
       </c>
@@ -1509,8 +1818,8 @@
       </c>
     </row>
     <row r="23" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A23" s="7" t="s">
-        <v>72</v>
+      <c r="A23" s="5" t="s">
+        <v>73</v>
       </c>
       <c r="B23" s="1" t="s">
         <v>37</v>
@@ -1518,7 +1827,7 @@
       <c r="C23" s="1" t="s">
         <v>24</v>
       </c>
-      <c r="D23" s="7" t="s">
+      <c r="D23" s="5" t="s">
         <v>38</v>
       </c>
       <c r="E23" s="1">
@@ -1534,7 +1843,7 @@
         <f t="shared" si="0"/>
         <v>9</v>
       </c>
-      <c r="I23" s="9">
+      <c r="I23" s="7">
         <f t="shared" si="1"/>
         <v>2.7777777777777781</v>
       </c>
@@ -1547,8 +1856,8 @@
       </c>
     </row>
     <row r="24" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A24" s="7" t="s">
-        <v>73</v>
+      <c r="A24" s="5" t="s">
+        <v>74</v>
       </c>
       <c r="B24" s="1" t="s">
         <v>39</v>
@@ -1556,7 +1865,7 @@
       <c r="C24" s="1" t="s">
         <v>18</v>
       </c>
-      <c r="D24" s="7" t="s">
+      <c r="D24" s="5" t="s">
         <v>40</v>
       </c>
       <c r="E24" s="1">
@@ -1572,7 +1881,7 @@
         <f t="shared" si="0"/>
         <v>13</v>
       </c>
-      <c r="I24" s="9">
+      <c r="I24" s="7">
         <f t="shared" si="1"/>
         <v>5.4444444444444455</v>
       </c>
@@ -1585,8 +1894,8 @@
       </c>
     </row>
     <row r="25" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A25" s="7" t="s">
-        <v>74</v>
+      <c r="A25" s="5" t="s">
+        <v>75</v>
       </c>
       <c r="B25" s="1" t="s">
         <v>41</v>
@@ -1594,8 +1903,8 @@
       <c r="C25" s="1" t="s">
         <v>24</v>
       </c>
-      <c r="D25" s="7" t="s">
-        <v>72</v>
+      <c r="D25" s="5" t="s">
+        <v>73</v>
       </c>
       <c r="E25" s="1">
         <v>6</v>
@@ -1610,7 +1919,7 @@
         <f t="shared" si="0"/>
         <v>9</v>
       </c>
-      <c r="I25" s="9">
+      <c r="I25" s="7">
         <f t="shared" si="1"/>
         <v>2.7777777777777781</v>
       </c>
@@ -1623,8 +1932,8 @@
       </c>
     </row>
     <row r="26" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A26" s="7" t="s">
-        <v>59</v>
+      <c r="A26" s="5" t="s">
+        <v>60</v>
       </c>
       <c r="B26" s="1" t="s">
         <v>42</v>
@@ -1632,7 +1941,7 @@
       <c r="C26" s="1" t="s">
         <v>18</v>
       </c>
-      <c r="D26" s="7" t="s">
+      <c r="D26" s="5" t="s">
         <v>43</v>
       </c>
       <c r="E26" s="1">
@@ -1648,7 +1957,7 @@
         <f t="shared" si="0"/>
         <v>17</v>
       </c>
-      <c r="I26" s="9">
+      <c r="I26" s="7">
         <f t="shared" si="1"/>
         <v>5.4444444444444455</v>
       </c>
@@ -1661,12 +1970,12 @@
       </c>
     </row>
     <row r="27" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A27" s="7" t="s">
+      <c r="A27" s="5" t="s">
         <v>44</v>
       </c>
       <c r="B27" s="1"/>
       <c r="C27" s="1"/>
-      <c r="D27" s="7"/>
+      <c r="D27" s="5"/>
       <c r="E27" s="1">
         <f>SUM(E2:E26)</f>
         <v>266</v>
@@ -1702,9 +2011,501 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{685DC2EE-ABFC-4F6B-8328-3A720D4D5FD0}">
-  <dimension ref="A1"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
-  <sheetData/>
+  <dimension ref="A1:G38"/>
+  <sheetFormatPr defaultColWidth="42" defaultRowHeight="18.75" x14ac:dyDescent="0.25"/>
+  <cols>
+    <col min="1" max="3" width="42" style="4"/>
+    <col min="4" max="4" width="23.7109375" style="4" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="24.85546875" style="4" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="26.28515625" style="4" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="30.85546875" style="4" bestFit="1" customWidth="1"/>
+    <col min="8" max="16384" width="42" style="4"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:3" s="10" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A1" s="9" t="s">
+        <v>91</v>
+      </c>
+      <c r="B1" s="9" t="s">
+        <v>92</v>
+      </c>
+      <c r="C1" s="9" t="s">
+        <v>93</v>
+      </c>
+    </row>
+    <row r="2" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A2" s="11" t="s">
+        <v>83</v>
+      </c>
+      <c r="B2" s="12"/>
+      <c r="C2" s="13"/>
+    </row>
+    <row r="3" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A3" s="14" t="s">
+        <v>84</v>
+      </c>
+      <c r="B3" s="15"/>
+      <c r="C3" s="16"/>
+    </row>
+    <row r="4" spans="1:3" ht="56.25" x14ac:dyDescent="0.25">
+      <c r="A4" s="1" t="s">
+        <v>85</v>
+      </c>
+      <c r="B4" s="1" t="s">
+        <v>86</v>
+      </c>
+      <c r="C4" s="1" t="s">
+        <v>87</v>
+      </c>
+    </row>
+    <row r="5" spans="1:3" ht="37.5" x14ac:dyDescent="0.25">
+      <c r="A5" s="1" t="s">
+        <v>88</v>
+      </c>
+      <c r="B5" s="1">
+        <f>'Оценки пакетов ИСР'!H2+'Оценки пакетов ИСР'!H9+'Оценки пакетов ИСР'!H11+'Оценки пакетов ИСР'!H12+'Оценки пакетов ИСР'!H13+'Оценки пакетов ИСР'!H14+'Оценки пакетов ИСР'!H15+'Оценки пакетов ИСР'!H17+'Оценки пакетов ИСР'!H18+'Оценки пакетов ИСР'!H23+'Оценки пакетов ИСР'!H24+'Оценки пакетов ИСР'!H26</f>
+        <v>197</v>
+      </c>
+      <c r="C5" s="1" t="s">
+        <v>94</v>
+      </c>
+    </row>
+    <row r="6" spans="1:3" ht="37.5" x14ac:dyDescent="0.25">
+      <c r="A6" s="1" t="s">
+        <v>89</v>
+      </c>
+      <c r="B6" s="7">
+        <f>'Оценки пакетов ИСР'!I2+'Оценки пакетов ИСР'!I9+'Оценки пакетов ИСР'!I11+'Оценки пакетов ИСР'!I12+'Оценки пакетов ИСР'!I13+'Оценки пакетов ИСР'!I14+'Оценки пакетов ИСР'!I15+'Оценки пакетов ИСР'!I17+'Оценки пакетов ИСР'!I18+'Оценки пакетов ИСР'!I23+'Оценки пакетов ИСР'!I24+'Оценки пакетов ИСР'!I26</f>
+        <v>71.8888888888889</v>
+      </c>
+      <c r="C6" s="1" t="s">
+        <v>95</v>
+      </c>
+    </row>
+    <row r="7" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A7" s="1" t="s">
+        <v>90</v>
+      </c>
+      <c r="B7" s="1">
+        <f>SQRT(B6)</f>
+        <v>8.4787315613179377</v>
+      </c>
+      <c r="C7" s="1"/>
+    </row>
+    <row r="8" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A8" s="1"/>
+      <c r="B8" s="1"/>
+      <c r="C8" s="1"/>
+    </row>
+    <row r="10" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A10" s="17" t="s">
+        <v>96</v>
+      </c>
+      <c r="B10" s="17"/>
+      <c r="C10" s="17"/>
+    </row>
+    <row r="11" spans="1:3" ht="37.5" x14ac:dyDescent="0.25">
+      <c r="A11" s="1" t="s">
+        <v>100</v>
+      </c>
+      <c r="B11" s="1">
+        <v>215</v>
+      </c>
+      <c r="C11" s="1" t="s">
+        <v>97</v>
+      </c>
+    </row>
+    <row r="12" spans="1:3" ht="37.5" x14ac:dyDescent="0.25">
+      <c r="A12" s="1" t="s">
+        <v>101</v>
+      </c>
+      <c r="B12" s="1">
+        <f>B5</f>
+        <v>197</v>
+      </c>
+      <c r="C12" s="1"/>
+    </row>
+    <row r="13" spans="1:3" ht="37.5" x14ac:dyDescent="0.25">
+      <c r="A13" s="1" t="s">
+        <v>102</v>
+      </c>
+      <c r="B13" s="1">
+        <f>(B11 - B12) / B7</f>
+        <v>2.1229590617210286</v>
+      </c>
+      <c r="C13" s="1" t="s">
+        <v>104</v>
+      </c>
+    </row>
+    <row r="14" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A14" s="1" t="s">
+        <v>103</v>
+      </c>
+      <c r="B14" s="18">
+        <f>_xlfn.NORM.S.DIST(B13, TRUE)</f>
+        <v>0.98312135874036699</v>
+      </c>
+      <c r="C14" s="1"/>
+    </row>
+    <row r="15" spans="1:3" ht="56.25" x14ac:dyDescent="0.25">
+      <c r="A15" s="1" t="s">
+        <v>98</v>
+      </c>
+      <c r="B15" s="19" t="s">
+        <v>99</v>
+      </c>
+      <c r="C15" s="20"/>
+    </row>
+    <row r="18" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A18" s="17" t="s">
+        <v>105</v>
+      </c>
+      <c r="B18" s="17"/>
+      <c r="C18" s="17"/>
+    </row>
+    <row r="19" spans="1:7" ht="37.5" x14ac:dyDescent="0.25">
+      <c r="A19" s="1" t="s">
+        <v>106</v>
+      </c>
+      <c r="B19" s="1">
+        <v>420</v>
+      </c>
+      <c r="C19" s="1" t="s">
+        <v>112</v>
+      </c>
+    </row>
+    <row r="20" spans="1:7" ht="37.5" x14ac:dyDescent="0.25">
+      <c r="A20" s="1" t="s">
+        <v>107</v>
+      </c>
+      <c r="B20" s="1">
+        <f>'Оценки пакетов ИСР'!H27</f>
+        <v>387</v>
+      </c>
+      <c r="C20" s="1" t="s">
+        <v>113</v>
+      </c>
+    </row>
+    <row r="21" spans="1:7" ht="37.5" x14ac:dyDescent="0.25">
+      <c r="A21" s="1" t="s">
+        <v>108</v>
+      </c>
+      <c r="B21" s="1">
+        <f>B19 - B20</f>
+        <v>33</v>
+      </c>
+      <c r="C21" s="1" t="s">
+        <v>114</v>
+      </c>
+    </row>
+    <row r="22" spans="1:7" ht="37.5" x14ac:dyDescent="0.25">
+      <c r="A22" s="1" t="s">
+        <v>109</v>
+      </c>
+      <c r="B22" s="1">
+        <v>222600</v>
+      </c>
+      <c r="C22" s="1" t="s">
+        <v>115</v>
+      </c>
+    </row>
+    <row r="23" spans="1:7" ht="37.5" x14ac:dyDescent="0.25">
+      <c r="A23" s="1" t="s">
+        <v>110</v>
+      </c>
+      <c r="B23" s="3">
+        <f>'Оценки пакетов ИСР'!K27</f>
+        <v>209850</v>
+      </c>
+      <c r="C23" s="1" t="s">
+        <v>116</v>
+      </c>
+    </row>
+    <row r="24" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A24" s="1" t="s">
+        <v>111</v>
+      </c>
+      <c r="B24" s="3">
+        <f>B22 - B23</f>
+        <v>12750</v>
+      </c>
+      <c r="C24" s="1" t="s">
+        <v>117</v>
+      </c>
+    </row>
+    <row r="27" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A27" s="21" t="s">
+        <v>118</v>
+      </c>
+      <c r="B27" s="22"/>
+      <c r="C27" s="22"/>
+      <c r="D27" s="22"/>
+      <c r="E27" s="22"/>
+      <c r="F27" s="22"/>
+      <c r="G27" s="23"/>
+    </row>
+    <row r="28" spans="1:7" s="10" customFormat="1" ht="37.5" x14ac:dyDescent="0.25">
+      <c r="A28" s="24" t="s">
+        <v>119</v>
+      </c>
+      <c r="B28" s="24" t="s">
+        <v>120</v>
+      </c>
+      <c r="C28" s="24" t="s">
+        <v>136</v>
+      </c>
+      <c r="D28" s="24" t="s">
+        <v>137</v>
+      </c>
+      <c r="E28" s="24" t="s">
+        <v>138</v>
+      </c>
+      <c r="F28" s="24" t="s">
+        <v>139</v>
+      </c>
+      <c r="G28" s="24" t="s">
+        <v>140</v>
+      </c>
+    </row>
+    <row r="29" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A29" s="25" t="s">
+        <v>121</v>
+      </c>
+      <c r="B29" s="24" t="s">
+        <v>1</v>
+      </c>
+      <c r="C29" s="24" t="s">
+        <v>142</v>
+      </c>
+      <c r="D29" s="24" t="s">
+        <v>122</v>
+      </c>
+      <c r="E29" s="24" t="s">
+        <v>123</v>
+      </c>
+      <c r="F29" s="24" t="s">
+        <v>124</v>
+      </c>
+      <c r="G29" s="24" t="s">
+        <v>125</v>
+      </c>
+    </row>
+    <row r="30" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A30" s="26" t="s">
+        <v>53</v>
+      </c>
+      <c r="B30" s="27" t="s">
+        <v>17</v>
+      </c>
+      <c r="C30" s="27">
+        <v>15</v>
+      </c>
+      <c r="D30" s="27">
+        <v>0</v>
+      </c>
+      <c r="E30" s="27">
+        <v>4</v>
+      </c>
+      <c r="F30" s="27" t="s">
+        <v>126</v>
+      </c>
+      <c r="G30" s="27" t="s">
+        <v>126</v>
+      </c>
+    </row>
+    <row r="31" spans="1:7" ht="37.5" x14ac:dyDescent="0.25">
+      <c r="A31" s="26" t="s">
+        <v>52</v>
+      </c>
+      <c r="B31" s="27" t="s">
+        <v>9</v>
+      </c>
+      <c r="C31" s="27">
+        <v>17</v>
+      </c>
+      <c r="D31" s="27">
+        <v>19</v>
+      </c>
+      <c r="E31" s="27">
+        <v>24</v>
+      </c>
+      <c r="F31" s="27" t="s">
+        <v>127</v>
+      </c>
+      <c r="G31" s="27" t="s">
+        <v>127</v>
+      </c>
+    </row>
+    <row r="32" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A32" s="26" t="s">
+        <v>55</v>
+      </c>
+      <c r="B32" s="27" t="s">
+        <v>11</v>
+      </c>
+      <c r="C32" s="27">
+        <v>11</v>
+      </c>
+      <c r="D32" s="27">
+        <v>19</v>
+      </c>
+      <c r="E32" s="27">
+        <v>30</v>
+      </c>
+      <c r="F32" s="27" t="s">
+        <v>128</v>
+      </c>
+      <c r="G32" s="27" t="s">
+        <v>128</v>
+      </c>
+    </row>
+    <row r="33" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A33" s="26" t="s">
+        <v>57</v>
+      </c>
+      <c r="B33" s="27" t="s">
+        <v>12</v>
+      </c>
+      <c r="C33" s="27">
+        <v>15</v>
+      </c>
+      <c r="D33" s="27">
+        <v>19</v>
+      </c>
+      <c r="E33" s="27">
+        <v>26</v>
+      </c>
+      <c r="F33" s="27" t="s">
+        <v>129</v>
+      </c>
+      <c r="G33" s="27" t="s">
+        <v>129</v>
+      </c>
+    </row>
+    <row r="34" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A34" s="26" t="s">
+        <v>141</v>
+      </c>
+      <c r="B34" s="27" t="s">
+        <v>130</v>
+      </c>
+      <c r="C34" s="27">
+        <v>30</v>
+      </c>
+      <c r="D34" s="27">
+        <v>38</v>
+      </c>
+      <c r="E34" s="27">
+        <v>51</v>
+      </c>
+      <c r="F34" s="27" t="s">
+        <v>131</v>
+      </c>
+      <c r="G34" s="27" t="s">
+        <v>131</v>
+      </c>
+    </row>
+    <row r="35" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A35" s="26" t="s">
+        <v>67</v>
+      </c>
+      <c r="B35" s="27" t="s">
+        <v>132</v>
+      </c>
+      <c r="C35" s="27">
+        <v>15</v>
+      </c>
+      <c r="D35" s="27">
+        <v>116</v>
+      </c>
+      <c r="E35" s="27">
+        <v>133</v>
+      </c>
+      <c r="F35" s="27" t="s">
+        <v>133</v>
+      </c>
+      <c r="G35" s="27" t="s">
+        <v>133</v>
+      </c>
+    </row>
+    <row r="36" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A36" s="26" t="s">
+        <v>54</v>
+      </c>
+      <c r="B36" s="27" t="s">
+        <v>33</v>
+      </c>
+      <c r="C36" s="27">
+        <v>13</v>
+      </c>
+      <c r="D36" s="27">
+        <v>136</v>
+      </c>
+      <c r="E36" s="27">
+        <v>158</v>
+      </c>
+      <c r="F36" s="27" t="s">
+        <v>134</v>
+      </c>
+      <c r="G36" s="27" t="s">
+        <v>134</v>
+      </c>
+    </row>
+    <row r="37" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A37" s="26" t="s">
+        <v>71</v>
+      </c>
+      <c r="B37" s="27" t="s">
+        <v>35</v>
+      </c>
+      <c r="C37" s="27">
+        <v>9</v>
+      </c>
+      <c r="D37" s="27">
+        <v>116</v>
+      </c>
+      <c r="E37" s="27">
+        <v>135</v>
+      </c>
+      <c r="F37" s="27" t="s">
+        <v>135</v>
+      </c>
+      <c r="G37" s="27" t="s">
+        <v>135</v>
+      </c>
+    </row>
+    <row r="38" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A38" s="26" t="s">
+        <v>72</v>
+      </c>
+      <c r="B38" s="27" t="s">
+        <v>36</v>
+      </c>
+      <c r="C38" s="27">
+        <v>9</v>
+      </c>
+      <c r="D38" s="27">
+        <v>116</v>
+      </c>
+      <c r="E38" s="27">
+        <v>135</v>
+      </c>
+      <c r="F38" s="27" t="s">
+        <v>135</v>
+      </c>
+      <c r="G38" s="27" t="s">
+        <v>135</v>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="5">
+    <mergeCell ref="A2:C2"/>
+    <mergeCell ref="A10:C10"/>
+    <mergeCell ref="A3:C3"/>
+    <mergeCell ref="A18:C18"/>
+    <mergeCell ref="A27:G27"/>
+  </mergeCells>
+  <phoneticPr fontId="3" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
docs: formatting has been corrected
</commit_message>
<xml_diff>
--- a/сводная таблица оценок и PERT.xlsx
+++ b/сводная таблица оценок и PERT.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/1f1cfff57e867f98/ВГУ/4 курс - 7 семестр/Управление проектами/photo-studio/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="353" documentId="11_AD4DF75460589B3ACB72848187DB6FA05ADEDD8E" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{59DEC8DC-2621-486D-A258-F8DC841BE7D4}"/>
+  <xr:revisionPtr revIDLastSave="370" documentId="11_AD4DF75460589B3ACB72848187DB6FA05ADEDD8E" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{E417D0EA-7983-4ED0-BFCF-3E7DB2F2AD09}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -472,8 +472,9 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <numFmts count="1">
+  <numFmts count="2">
     <numFmt numFmtId="6" formatCode="#,##0\ &quot;₽&quot;;[Red]\-#,##0\ &quot;₽&quot;"/>
+    <numFmt numFmtId="175" formatCode="0.000"/>
   </numFmts>
   <fonts count="5" x14ac:knownFonts="1">
     <font>
@@ -623,6 +624,9 @@
     <xf numFmtId="49" fontId="2" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="175" fontId="2" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
     <xf numFmtId="2" fontId="2" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
@@ -659,12 +663,6 @@
     <xf numFmtId="9" fontId="2" fillId="0" borderId="1" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="2" fillId="3" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
@@ -685,6 +683,9 @@
     </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="2">
@@ -984,38 +985,38 @@
     <col min="12" max="16384" width="9.140625" style="4"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:11" s="10" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A1" s="8" t="s">
+    <row r="1" spans="1:11" s="11" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A1" s="9" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="9" t="s">
+      <c r="B1" s="10" t="s">
         <v>1</v>
       </c>
-      <c r="C1" s="9" t="s">
+      <c r="C1" s="10" t="s">
         <v>2</v>
       </c>
-      <c r="D1" s="8" t="s">
+      <c r="D1" s="9" t="s">
         <v>3</v>
       </c>
-      <c r="E1" s="9" t="s">
+      <c r="E1" s="10" t="s">
         <v>45</v>
       </c>
-      <c r="F1" s="9" t="s">
+      <c r="F1" s="10" t="s">
         <v>49</v>
       </c>
-      <c r="G1" s="9" t="s">
+      <c r="G1" s="10" t="s">
         <v>46</v>
       </c>
-      <c r="H1" s="9" t="s">
+      <c r="H1" s="10" t="s">
         <v>48</v>
       </c>
-      <c r="I1" s="8" t="s">
+      <c r="I1" s="9" t="s">
         <v>47</v>
       </c>
-      <c r="J1" s="9" t="s">
+      <c r="J1" s="10" t="s">
         <v>4</v>
       </c>
-      <c r="K1" s="9" t="s">
+      <c r="K1" s="10" t="s">
         <v>5</v>
       </c>
     </row>
@@ -1045,7 +1046,7 @@
         <f>(E2 + 4*F2 + G2) / 6</f>
         <v>19</v>
       </c>
-      <c r="I2" s="7">
+      <c r="I2" s="8">
         <f>((G2 - E2) / 6)^2</f>
         <v>5.4444444444444455</v>
       </c>
@@ -1083,7 +1084,7 @@
         <f t="shared" ref="H3:H27" si="0">(E3 + 4*F3 + G3) / 6</f>
         <v>17</v>
       </c>
-      <c r="I3" s="7">
+      <c r="I3" s="8">
         <f t="shared" ref="I3:I26" si="1">((G3 - E3) / 6)^2</f>
         <v>5.4444444444444455</v>
       </c>
@@ -1121,7 +1122,7 @@
         <f t="shared" si="0"/>
         <v>11</v>
       </c>
-      <c r="I4" s="7">
+      <c r="I4" s="8">
         <f t="shared" si="1"/>
         <v>2.7777777777777781</v>
       </c>
@@ -1159,7 +1160,7 @@
         <f t="shared" si="0"/>
         <v>15</v>
       </c>
-      <c r="I5" s="7">
+      <c r="I5" s="8">
         <f t="shared" si="1"/>
         <v>5.4444444444444455</v>
       </c>
@@ -1197,7 +1198,7 @@
         <f t="shared" si="0"/>
         <v>15</v>
       </c>
-      <c r="I6" s="7">
+      <c r="I6" s="8">
         <f t="shared" si="1"/>
         <v>5.4444444444444455</v>
       </c>
@@ -1235,7 +1236,7 @@
         <f t="shared" si="0"/>
         <v>17</v>
       </c>
-      <c r="I7" s="7">
+      <c r="I7" s="8">
         <f t="shared" si="1"/>
         <v>5.4444444444444455</v>
       </c>
@@ -1273,7 +1274,7 @@
         <f t="shared" si="0"/>
         <v>15</v>
       </c>
-      <c r="I8" s="7">
+      <c r="I8" s="8">
         <f t="shared" si="1"/>
         <v>5.4444444444444455</v>
       </c>
@@ -1311,7 +1312,7 @@
         <f t="shared" si="0"/>
         <v>19</v>
       </c>
-      <c r="I9" s="7">
+      <c r="I9" s="8">
         <f t="shared" si="1"/>
         <v>5.4444444444444455</v>
       </c>
@@ -1349,7 +1350,7 @@
         <f t="shared" si="0"/>
         <v>30</v>
       </c>
-      <c r="I10" s="7">
+      <c r="I10" s="8">
         <f t="shared" si="1"/>
         <v>16</v>
       </c>
@@ -1387,7 +1388,7 @@
         <f t="shared" si="0"/>
         <v>15</v>
       </c>
-      <c r="I11" s="7">
+      <c r="I11" s="8">
         <f t="shared" si="1"/>
         <v>5.4444444444444455</v>
       </c>
@@ -1425,7 +1426,7 @@
         <f t="shared" si="0"/>
         <v>13</v>
       </c>
-      <c r="I12" s="7">
+      <c r="I12" s="8">
         <f t="shared" si="1"/>
         <v>5.4444444444444455</v>
       </c>
@@ -1463,7 +1464,7 @@
         <f t="shared" si="0"/>
         <v>15</v>
       </c>
-      <c r="I13" s="7">
+      <c r="I13" s="8">
         <f t="shared" si="1"/>
         <v>5.4444444444444455</v>
       </c>
@@ -1501,7 +1502,7 @@
         <f t="shared" si="0"/>
         <v>17</v>
       </c>
-      <c r="I14" s="7">
+      <c r="I14" s="8">
         <f t="shared" si="1"/>
         <v>5.4444444444444455</v>
       </c>
@@ -1539,7 +1540,7 @@
         <f t="shared" si="0"/>
         <v>23</v>
       </c>
-      <c r="I15" s="7">
+      <c r="I15" s="8">
         <f t="shared" si="1"/>
         <v>9</v>
       </c>
@@ -1577,7 +1578,7 @@
         <f t="shared" si="0"/>
         <v>15</v>
       </c>
-      <c r="I16" s="7">
+      <c r="I16" s="8">
         <f t="shared" si="1"/>
         <v>5.4444444444444455</v>
       </c>
@@ -1615,7 +1616,7 @@
         <f t="shared" si="0"/>
         <v>20</v>
       </c>
-      <c r="I17" s="7">
+      <c r="I17" s="8">
         <f t="shared" si="1"/>
         <v>11.111111111111112</v>
       </c>
@@ -1653,7 +1654,7 @@
         <f t="shared" si="0"/>
         <v>17</v>
       </c>
-      <c r="I18" s="7">
+      <c r="I18" s="8">
         <f t="shared" si="1"/>
         <v>5.4444444444444455</v>
       </c>
@@ -1691,7 +1692,7 @@
         <f t="shared" si="0"/>
         <v>13</v>
       </c>
-      <c r="I19" s="7">
+      <c r="I19" s="8">
         <f t="shared" si="1"/>
         <v>5.4444444444444455</v>
       </c>
@@ -1729,7 +1730,7 @@
         <f t="shared" si="0"/>
         <v>15</v>
       </c>
-      <c r="I20" s="7">
+      <c r="I20" s="8">
         <f t="shared" si="1"/>
         <v>5.4444444444444455</v>
       </c>
@@ -1767,7 +1768,7 @@
         <f t="shared" si="0"/>
         <v>9</v>
       </c>
-      <c r="I21" s="7">
+      <c r="I21" s="8">
         <f t="shared" si="1"/>
         <v>2.7777777777777781</v>
       </c>
@@ -1805,7 +1806,7 @@
         <f t="shared" si="0"/>
         <v>9</v>
       </c>
-      <c r="I22" s="7">
+      <c r="I22" s="8">
         <f t="shared" si="1"/>
         <v>2.7777777777777781</v>
       </c>
@@ -1843,7 +1844,7 @@
         <f t="shared" si="0"/>
         <v>9</v>
       </c>
-      <c r="I23" s="7">
+      <c r="I23" s="8">
         <f t="shared" si="1"/>
         <v>2.7777777777777781</v>
       </c>
@@ -1881,7 +1882,7 @@
         <f t="shared" si="0"/>
         <v>13</v>
       </c>
-      <c r="I24" s="7">
+      <c r="I24" s="8">
         <f t="shared" si="1"/>
         <v>5.4444444444444455</v>
       </c>
@@ -1919,7 +1920,7 @@
         <f t="shared" si="0"/>
         <v>9</v>
       </c>
-      <c r="I25" s="7">
+      <c r="I25" s="8">
         <f t="shared" si="1"/>
         <v>2.7777777777777781</v>
       </c>
@@ -1957,7 +1958,7 @@
         <f t="shared" si="0"/>
         <v>17</v>
       </c>
-      <c r="I26" s="7">
+      <c r="I26" s="8">
         <f t="shared" si="1"/>
         <v>5.4444444444444455</v>
       </c>
@@ -1992,7 +1993,7 @@
         <f>SUM(H2:H26)</f>
         <v>387</v>
       </c>
-      <c r="I27" s="7" t="s">
+      <c r="I27" s="8" t="s">
         <v>8</v>
       </c>
       <c r="J27" s="1" t="s">
@@ -2022,30 +2023,30 @@
     <col min="8" max="16384" width="42" style="4"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" s="10" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A1" s="9" t="s">
+    <row r="1" spans="1:3" s="11" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A1" s="10" t="s">
         <v>91</v>
       </c>
-      <c r="B1" s="9" t="s">
+      <c r="B1" s="10" t="s">
         <v>92</v>
       </c>
-      <c r="C1" s="9" t="s">
+      <c r="C1" s="10" t="s">
         <v>93</v>
       </c>
     </row>
     <row r="2" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A2" s="11" t="s">
+      <c r="A2" s="12" t="s">
         <v>83</v>
       </c>
-      <c r="B2" s="12"/>
-      <c r="C2" s="13"/>
+      <c r="B2" s="13"/>
+      <c r="C2" s="14"/>
     </row>
     <row r="3" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A3" s="14" t="s">
+      <c r="A3" s="15" t="s">
         <v>84</v>
       </c>
-      <c r="B3" s="15"/>
-      <c r="C3" s="16"/>
+      <c r="B3" s="16"/>
+      <c r="C3" s="17"/>
     </row>
     <row r="4" spans="1:3" ht="56.25" x14ac:dyDescent="0.25">
       <c r="A4" s="1" t="s">
@@ -2074,7 +2075,7 @@
       <c r="A6" s="1" t="s">
         <v>89</v>
       </c>
-      <c r="B6" s="7">
+      <c r="B6" s="8">
         <f>'Оценки пакетов ИСР'!I2+'Оценки пакетов ИСР'!I9+'Оценки пакетов ИСР'!I11+'Оценки пакетов ИСР'!I12+'Оценки пакетов ИСР'!I13+'Оценки пакетов ИСР'!I14+'Оценки пакетов ИСР'!I15+'Оценки пакетов ИСР'!I17+'Оценки пакетов ИСР'!I18+'Оценки пакетов ИСР'!I23+'Оценки пакетов ИСР'!I24+'Оценки пакетов ИСР'!I26</f>
         <v>71.8888888888889</v>
       </c>
@@ -2086,23 +2087,23 @@
       <c r="A7" s="1" t="s">
         <v>90</v>
       </c>
-      <c r="B7" s="1">
+      <c r="B7" s="7">
         <f>SQRT(B6)</f>
         <v>8.4787315613179377</v>
       </c>
       <c r="C7" s="1"/>
     </row>
     <row r="8" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A8" s="1"/>
-      <c r="B8" s="1"/>
-      <c r="C8" s="1"/>
+      <c r="A8" s="27"/>
+      <c r="B8" s="27"/>
+      <c r="C8" s="27"/>
     </row>
     <row r="10" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A10" s="17" t="s">
+      <c r="A10" s="18" t="s">
         <v>96</v>
       </c>
-      <c r="B10" s="17"/>
-      <c r="C10" s="17"/>
+      <c r="B10" s="18"/>
+      <c r="C10" s="18"/>
     </row>
     <row r="11" spans="1:3" ht="37.5" x14ac:dyDescent="0.25">
       <c r="A11" s="1" t="s">
@@ -2129,7 +2130,7 @@
       <c r="A13" s="1" t="s">
         <v>102</v>
       </c>
-      <c r="B13" s="1">
+      <c r="B13" s="7">
         <f>(B11 - B12) / B7</f>
         <v>2.1229590617210286</v>
       </c>
@@ -2141,27 +2142,27 @@
       <c r="A14" s="1" t="s">
         <v>103</v>
       </c>
-      <c r="B14" s="18">
+      <c r="B14" s="19">
         <f>_xlfn.NORM.S.DIST(B13, TRUE)</f>
         <v>0.98312135874036699</v>
       </c>
       <c r="C14" s="1"/>
     </row>
-    <row r="15" spans="1:3" ht="56.25" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:3" ht="56.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A15" s="1" t="s">
         <v>98</v>
       </c>
-      <c r="B15" s="19" t="s">
+      <c r="B15" s="15" t="s">
         <v>99</v>
       </c>
-      <c r="C15" s="20"/>
+      <c r="C15" s="17"/>
     </row>
     <row r="18" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A18" s="17" t="s">
+      <c r="A18" s="18" t="s">
         <v>105</v>
       </c>
-      <c r="B18" s="17"/>
-      <c r="C18" s="17"/>
+      <c r="B18" s="18"/>
+      <c r="C18" s="18"/>
     </row>
     <row r="19" spans="1:7" ht="37.5" x14ac:dyDescent="0.25">
       <c r="A19" s="1" t="s">
@@ -2234,274 +2235,275 @@
       </c>
     </row>
     <row r="27" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A27" s="21" t="s">
+      <c r="A27" s="20" t="s">
         <v>118</v>
       </c>
-      <c r="B27" s="22"/>
-      <c r="C27" s="22"/>
-      <c r="D27" s="22"/>
-      <c r="E27" s="22"/>
-      <c r="F27" s="22"/>
-      <c r="G27" s="23"/>
-    </row>
-    <row r="28" spans="1:7" s="10" customFormat="1" ht="37.5" x14ac:dyDescent="0.25">
-      <c r="A28" s="24" t="s">
+      <c r="B27" s="21"/>
+      <c r="C27" s="21"/>
+      <c r="D27" s="21"/>
+      <c r="E27" s="21"/>
+      <c r="F27" s="21"/>
+      <c r="G27" s="22"/>
+    </row>
+    <row r="28" spans="1:7" s="11" customFormat="1" ht="37.5" x14ac:dyDescent="0.25">
+      <c r="A28" s="23" t="s">
         <v>119</v>
       </c>
-      <c r="B28" s="24" t="s">
+      <c r="B28" s="23" t="s">
         <v>120</v>
       </c>
-      <c r="C28" s="24" t="s">
+      <c r="C28" s="23" t="s">
         <v>136</v>
       </c>
-      <c r="D28" s="24" t="s">
+      <c r="D28" s="23" t="s">
         <v>137</v>
       </c>
-      <c r="E28" s="24" t="s">
+      <c r="E28" s="23" t="s">
         <v>138</v>
       </c>
-      <c r="F28" s="24" t="s">
+      <c r="F28" s="23" t="s">
         <v>139</v>
       </c>
-      <c r="G28" s="24" t="s">
+      <c r="G28" s="23" t="s">
         <v>140</v>
       </c>
     </row>
     <row r="29" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A29" s="25" t="s">
+      <c r="A29" s="24" t="s">
         <v>121</v>
       </c>
-      <c r="B29" s="24" t="s">
+      <c r="B29" s="23" t="s">
         <v>1</v>
       </c>
-      <c r="C29" s="24" t="s">
+      <c r="C29" s="23" t="s">
         <v>142</v>
       </c>
-      <c r="D29" s="24" t="s">
+      <c r="D29" s="23" t="s">
         <v>122</v>
       </c>
-      <c r="E29" s="24" t="s">
+      <c r="E29" s="23" t="s">
         <v>123</v>
       </c>
-      <c r="F29" s="24" t="s">
+      <c r="F29" s="23" t="s">
         <v>124</v>
       </c>
-      <c r="G29" s="24" t="s">
+      <c r="G29" s="23" t="s">
         <v>125</v>
       </c>
     </row>
     <row r="30" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A30" s="26" t="s">
+      <c r="A30" s="25" t="s">
         <v>53</v>
       </c>
-      <c r="B30" s="27" t="s">
+      <c r="B30" s="26" t="s">
         <v>17</v>
       </c>
-      <c r="C30" s="27">
+      <c r="C30" s="26">
         <v>15</v>
       </c>
-      <c r="D30" s="27">
+      <c r="D30" s="26">
         <v>0</v>
       </c>
-      <c r="E30" s="27">
+      <c r="E30" s="26">
         <v>4</v>
       </c>
-      <c r="F30" s="27" t="s">
+      <c r="F30" s="26" t="s">
         <v>126</v>
       </c>
-      <c r="G30" s="27" t="s">
+      <c r="G30" s="26" t="s">
         <v>126</v>
       </c>
     </row>
     <row r="31" spans="1:7" ht="37.5" x14ac:dyDescent="0.25">
-      <c r="A31" s="26" t="s">
+      <c r="A31" s="25" t="s">
         <v>52</v>
       </c>
-      <c r="B31" s="27" t="s">
+      <c r="B31" s="26" t="s">
         <v>9</v>
       </c>
-      <c r="C31" s="27">
+      <c r="C31" s="26">
         <v>17</v>
       </c>
-      <c r="D31" s="27">
+      <c r="D31" s="26">
         <v>19</v>
       </c>
-      <c r="E31" s="27">
+      <c r="E31" s="26">
         <v>24</v>
       </c>
-      <c r="F31" s="27" t="s">
+      <c r="F31" s="26" t="s">
         <v>127</v>
       </c>
-      <c r="G31" s="27" t="s">
+      <c r="G31" s="26" t="s">
         <v>127</v>
       </c>
     </row>
     <row r="32" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A32" s="26" t="s">
+      <c r="A32" s="25" t="s">
         <v>55</v>
       </c>
-      <c r="B32" s="27" t="s">
+      <c r="B32" s="26" t="s">
         <v>11</v>
       </c>
-      <c r="C32" s="27">
+      <c r="C32" s="26">
         <v>11</v>
       </c>
-      <c r="D32" s="27">
+      <c r="D32" s="26">
         <v>19</v>
       </c>
-      <c r="E32" s="27">
+      <c r="E32" s="26">
         <v>30</v>
       </c>
-      <c r="F32" s="27" t="s">
+      <c r="F32" s="26" t="s">
         <v>128</v>
       </c>
-      <c r="G32" s="27" t="s">
+      <c r="G32" s="26" t="s">
         <v>128</v>
       </c>
     </row>
     <row r="33" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A33" s="26" t="s">
+      <c r="A33" s="25" t="s">
         <v>57</v>
       </c>
-      <c r="B33" s="27" t="s">
+      <c r="B33" s="26" t="s">
         <v>12</v>
       </c>
-      <c r="C33" s="27">
+      <c r="C33" s="26">
         <v>15</v>
       </c>
-      <c r="D33" s="27">
+      <c r="D33" s="26">
         <v>19</v>
       </c>
-      <c r="E33" s="27">
+      <c r="E33" s="26">
         <v>26</v>
       </c>
-      <c r="F33" s="27" t="s">
+      <c r="F33" s="26" t="s">
         <v>129</v>
       </c>
-      <c r="G33" s="27" t="s">
+      <c r="G33" s="26" t="s">
         <v>129</v>
       </c>
     </row>
     <row r="34" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A34" s="26" t="s">
+      <c r="A34" s="25" t="s">
         <v>141</v>
       </c>
-      <c r="B34" s="27" t="s">
+      <c r="B34" s="26" t="s">
         <v>130</v>
       </c>
-      <c r="C34" s="27">
+      <c r="C34" s="26">
         <v>30</v>
       </c>
-      <c r="D34" s="27">
+      <c r="D34" s="26">
         <v>38</v>
       </c>
-      <c r="E34" s="27">
+      <c r="E34" s="26">
         <v>51</v>
       </c>
-      <c r="F34" s="27" t="s">
+      <c r="F34" s="26" t="s">
         <v>131</v>
       </c>
-      <c r="G34" s="27" t="s">
+      <c r="G34" s="26" t="s">
         <v>131</v>
       </c>
     </row>
     <row r="35" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A35" s="26" t="s">
+      <c r="A35" s="25" t="s">
         <v>67</v>
       </c>
-      <c r="B35" s="27" t="s">
+      <c r="B35" s="26" t="s">
         <v>132</v>
       </c>
-      <c r="C35" s="27">
+      <c r="C35" s="26">
         <v>15</v>
       </c>
-      <c r="D35" s="27">
+      <c r="D35" s="26">
         <v>116</v>
       </c>
-      <c r="E35" s="27">
+      <c r="E35" s="26">
         <v>133</v>
       </c>
-      <c r="F35" s="27" t="s">
+      <c r="F35" s="26" t="s">
         <v>133</v>
       </c>
-      <c r="G35" s="27" t="s">
+      <c r="G35" s="26" t="s">
         <v>133</v>
       </c>
     </row>
     <row r="36" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A36" s="26" t="s">
+      <c r="A36" s="25" t="s">
         <v>54</v>
       </c>
-      <c r="B36" s="27" t="s">
+      <c r="B36" s="26" t="s">
         <v>33</v>
       </c>
-      <c r="C36" s="27">
+      <c r="C36" s="26">
         <v>13</v>
       </c>
-      <c r="D36" s="27">
+      <c r="D36" s="26">
         <v>136</v>
       </c>
-      <c r="E36" s="27">
+      <c r="E36" s="26">
         <v>158</v>
       </c>
-      <c r="F36" s="27" t="s">
+      <c r="F36" s="26" t="s">
         <v>134</v>
       </c>
-      <c r="G36" s="27" t="s">
+      <c r="G36" s="26" t="s">
         <v>134</v>
       </c>
     </row>
     <row r="37" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A37" s="26" t="s">
+      <c r="A37" s="25" t="s">
         <v>71</v>
       </c>
-      <c r="B37" s="27" t="s">
+      <c r="B37" s="26" t="s">
         <v>35</v>
       </c>
-      <c r="C37" s="27">
+      <c r="C37" s="26">
         <v>9</v>
       </c>
-      <c r="D37" s="27">
+      <c r="D37" s="26">
         <v>116</v>
       </c>
-      <c r="E37" s="27">
+      <c r="E37" s="26">
         <v>135</v>
       </c>
-      <c r="F37" s="27" t="s">
+      <c r="F37" s="26" t="s">
         <v>135</v>
       </c>
-      <c r="G37" s="27" t="s">
+      <c r="G37" s="26" t="s">
         <v>135</v>
       </c>
     </row>
     <row r="38" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A38" s="26" t="s">
+      <c r="A38" s="25" t="s">
         <v>72</v>
       </c>
-      <c r="B38" s="27" t="s">
+      <c r="B38" s="26" t="s">
         <v>36</v>
       </c>
-      <c r="C38" s="27">
+      <c r="C38" s="26">
         <v>9</v>
       </c>
-      <c r="D38" s="27">
+      <c r="D38" s="26">
         <v>116</v>
       </c>
-      <c r="E38" s="27">
+      <c r="E38" s="26">
         <v>135</v>
       </c>
-      <c r="F38" s="27" t="s">
+      <c r="F38" s="26" t="s">
         <v>135</v>
       </c>
-      <c r="G38" s="27" t="s">
+      <c r="G38" s="26" t="s">
         <v>135</v>
       </c>
     </row>
   </sheetData>
-  <mergeCells count="5">
+  <mergeCells count="6">
     <mergeCell ref="A2:C2"/>
     <mergeCell ref="A10:C10"/>
     <mergeCell ref="A3:C3"/>
+    <mergeCell ref="B15:C15"/>
     <mergeCell ref="A18:C18"/>
     <mergeCell ref="A27:G27"/>
   </mergeCells>

</xml_diff>